<commit_message>
Split blueprint support task categories
</commit_message>
<xml_diff>
--- a/outputs/vc-pr26-project-task-doc-map-blueprints-github-links.xlsx
+++ b/outputs/vc-pr26-project-task-doc-map-blueprints-github-links.xlsx
@@ -2460,7 +2460,7 @@
       </c>
       <c r="C36" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D36" s="16">
@@ -2510,7 +2510,7 @@
       </c>
       <c r="C37" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D37" s="16">
@@ -2556,7 +2556,7 @@
       </c>
       <c r="C38" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D38" s="16">
@@ -2606,7 +2606,7 @@
       </c>
       <c r="C39" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D39" s="16">
@@ -2652,7 +2652,7 @@
       </c>
       <c r="C40" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D40" s="16">
@@ -2702,7 +2702,7 @@
       </c>
       <c r="C41" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D41" s="16">
@@ -2748,7 +2748,7 @@
       </c>
       <c r="C42" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D42" s="16">
@@ -2798,7 +2798,7 @@
       </c>
       <c r="C43" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D43" s="16">
@@ -2844,7 +2844,7 @@
       </c>
       <c r="C44" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D44" s="16">
@@ -2894,7 +2894,7 @@
       </c>
       <c r="C45" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D45" s="16">
@@ -2940,7 +2940,7 @@
       </c>
       <c r="C46" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D46" s="16">
@@ -2990,7 +2990,7 @@
       </c>
       <c r="C47" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D47" s="16">
@@ -3036,7 +3036,7 @@
       </c>
       <c r="C48" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D48" s="16">
@@ -3086,7 +3086,7 @@
       </c>
       <c r="C49" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D49" s="16">
@@ -3132,7 +3132,7 @@
       </c>
       <c r="C50" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D50" s="16">
@@ -3182,7 +3182,7 @@
       </c>
       <c r="C51" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D51" s="16">
@@ -3228,7 +3228,7 @@
       </c>
       <c r="C52" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D52" s="16">
@@ -3278,7 +3278,7 @@
       </c>
       <c r="C53" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D53" s="16">
@@ -3324,7 +3324,7 @@
       </c>
       <c r="C54" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D54" s="16">
@@ -3374,7 +3374,7 @@
       </c>
       <c r="C55" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D55" s="16">
@@ -3420,7 +3420,7 @@
       </c>
       <c r="C56" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Pipeline Management</t>
         </is>
       </c>
       <c r="D56" s="16">
@@ -3475,7 +3475,7 @@
       </c>
       <c r="C57" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Pipeline Management</t>
         </is>
       </c>
       <c r="D57" s="16">
@@ -3526,7 +3526,7 @@
       </c>
       <c r="C58" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D58" s="16">
@@ -3576,7 +3576,7 @@
       </c>
       <c r="C59" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D59" s="16">
@@ -3622,7 +3622,7 @@
       </c>
       <c r="C60" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D60" s="16">
@@ -3672,7 +3672,7 @@
       </c>
       <c r="C61" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D61" s="16">
@@ -3718,7 +3718,7 @@
       </c>
       <c r="C62" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D62" s="16">
@@ -3768,7 +3768,7 @@
       </c>
       <c r="C63" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D63" s="16">
@@ -3814,7 +3814,7 @@
       </c>
       <c r="C64" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D64" s="16">
@@ -3864,7 +3864,7 @@
       </c>
       <c r="C65" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D65" s="16">
@@ -3910,7 +3910,7 @@
       </c>
       <c r="C66" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D66" s="16">
@@ -3960,7 +3960,7 @@
       </c>
       <c r="C67" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D67" s="16">
@@ -4006,7 +4006,7 @@
       </c>
       <c r="C68" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D68" s="16">
@@ -4052,7 +4052,7 @@
       </c>
       <c r="C69" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D69" s="16">
@@ -4098,7 +4098,7 @@
       </c>
       <c r="C70" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D70" s="16">
@@ -4148,7 +4148,7 @@
       </c>
       <c r="C71" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D71" s="16">
@@ -4194,7 +4194,7 @@
       </c>
       <c r="C72" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D72" s="16">
@@ -4240,7 +4240,7 @@
       </c>
       <c r="C73" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D73" s="16">
@@ -4290,7 +4290,7 @@
       </c>
       <c r="C74" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D74" s="16">
@@ -4336,7 +4336,7 @@
       </c>
       <c r="C75" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D75" s="16">
@@ -4382,7 +4382,7 @@
       </c>
       <c r="C76" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D76" s="16">
@@ -4428,7 +4428,7 @@
       </c>
       <c r="C77" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D77" s="16">
@@ -4478,7 +4478,7 @@
       </c>
       <c r="C78" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D78" s="16">
@@ -4524,7 +4524,7 @@
       </c>
       <c r="C79" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D79" s="16">
@@ -4570,7 +4570,7 @@
       </c>
       <c r="C80" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D80" s="16">
@@ -10294,7 +10294,7 @@
       </c>
       <c r="C184" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Pipeline Management</t>
         </is>
       </c>
       <c r="D184" s="16">
@@ -10347,7 +10347,7 @@
       </c>
       <c r="C185" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Pipeline Management</t>
         </is>
       </c>
       <c r="D185" s="16">
@@ -10400,7 +10400,7 @@
       </c>
       <c r="C186" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Pipeline Management</t>
         </is>
       </c>
       <c r="D186" s="16">
@@ -10449,7 +10449,7 @@
       </c>
       <c r="C187" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D187" s="16">
@@ -10499,7 +10499,7 @@
       </c>
       <c r="C188" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D188" s="16">
@@ -10545,7 +10545,7 @@
       </c>
       <c r="C189" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D189" s="16">
@@ -10595,7 +10595,7 @@
       </c>
       <c r="C190" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D190" s="16">
@@ -10641,7 +10641,7 @@
       </c>
       <c r="C191" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Pipeline Management</t>
         </is>
       </c>
       <c r="D191" s="16">
@@ -10698,7 +10698,7 @@
       </c>
       <c r="C192" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Pipeline Management</t>
         </is>
       </c>
       <c r="D192" s="16">
@@ -10755,7 +10755,7 @@
       </c>
       <c r="C193" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Pipeline Management</t>
         </is>
       </c>
       <c r="D193" s="16">
@@ -10809,7 +10809,7 @@
       </c>
       <c r="C194" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Pipeline Management</t>
         </is>
       </c>
       <c r="D194" s="16">
@@ -10863,7 +10863,7 @@
       </c>
       <c r="C195" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D195" s="16">
@@ -10913,7 +10913,7 @@
       </c>
       <c r="C196" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D196" s="16">
@@ -10959,7 +10959,7 @@
       </c>
       <c r="C197" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D197" s="16">
@@ -11009,7 +11009,7 @@
       </c>
       <c r="C198" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="D198" s="16">
@@ -25062,7 +25062,7 @@
       </c>
       <c r="B26" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C26" s="16">
@@ -25082,7 +25082,7 @@
       </c>
       <c r="B27" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C27" s="16">
@@ -25102,7 +25102,7 @@
       </c>
       <c r="B28" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C28" s="16">
@@ -25122,7 +25122,7 @@
       </c>
       <c r="B29" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C29" s="16">
@@ -25142,7 +25142,7 @@
       </c>
       <c r="B30" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C30" s="16">
@@ -25162,7 +25162,7 @@
       </c>
       <c r="B31" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C31" s="16">
@@ -25182,7 +25182,7 @@
       </c>
       <c r="B32" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C32" s="16">
@@ -25202,7 +25202,7 @@
       </c>
       <c r="B33" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C33" s="16">
@@ -25222,7 +25222,7 @@
       </c>
       <c r="B34" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C34" s="16">
@@ -25242,7 +25242,7 @@
       </c>
       <c r="B35" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C35" s="16">
@@ -25262,7 +25262,7 @@
       </c>
       <c r="B36" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C36" s="16">
@@ -25282,7 +25282,7 @@
       </c>
       <c r="B37" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C37" s="16">
@@ -25302,7 +25302,7 @@
       </c>
       <c r="B38" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C38" s="16">
@@ -25322,7 +25322,7 @@
       </c>
       <c r="B39" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C39" s="16">
@@ -25342,7 +25342,7 @@
       </c>
       <c r="B40" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C40" s="16">
@@ -25362,7 +25362,7 @@
       </c>
       <c r="B41" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C41" s="16">
@@ -25382,7 +25382,7 @@
       </c>
       <c r="B42" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C42" s="16">
@@ -25402,7 +25402,7 @@
       </c>
       <c r="B43" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C43" s="16">
@@ -25422,7 +25422,7 @@
       </c>
       <c r="B44" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C44" s="16">
@@ -25442,7 +25442,7 @@
       </c>
       <c r="B45" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C45" s="16">
@@ -25462,7 +25462,7 @@
       </c>
       <c r="B46" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Pipeline Management</t>
         </is>
       </c>
       <c r="C46" s="16">
@@ -25482,7 +25482,7 @@
       </c>
       <c r="B47" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Pipeline Management</t>
         </is>
       </c>
       <c r="C47" s="16">
@@ -25502,7 +25502,7 @@
       </c>
       <c r="B48" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C48" s="16">
@@ -25522,7 +25522,7 @@
       </c>
       <c r="B49" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C49" s="16">
@@ -25542,7 +25542,7 @@
       </c>
       <c r="B50" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C50" s="16">
@@ -25562,7 +25562,7 @@
       </c>
       <c r="B51" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C51" s="16">
@@ -25582,7 +25582,7 @@
       </c>
       <c r="B52" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C52" s="16">
@@ -25602,7 +25602,7 @@
       </c>
       <c r="B53" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C53" s="16">
@@ -25622,7 +25622,7 @@
       </c>
       <c r="B54" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C54" s="16">
@@ -25642,7 +25642,7 @@
       </c>
       <c r="B55" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C55" s="16">
@@ -25662,7 +25662,7 @@
       </c>
       <c r="B56" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C56" s="16">
@@ -25682,7 +25682,7 @@
       </c>
       <c r="B57" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C57" s="16">
@@ -25702,7 +25702,7 @@
       </c>
       <c r="B58" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C58" s="16">
@@ -25722,7 +25722,7 @@
       </c>
       <c r="B59" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C59" s="16">
@@ -25742,7 +25742,7 @@
       </c>
       <c r="B60" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C60" s="16">
@@ -25762,7 +25762,7 @@
       </c>
       <c r="B61" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C61" s="16">
@@ -25782,7 +25782,7 @@
       </c>
       <c r="B62" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C62" s="16">
@@ -25802,7 +25802,7 @@
       </c>
       <c r="B63" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C63" s="16">
@@ -25822,7 +25822,7 @@
       </c>
       <c r="B64" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C64" s="16">
@@ -25842,7 +25842,7 @@
       </c>
       <c r="B65" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C65" s="16">
@@ -25862,7 +25862,7 @@
       </c>
       <c r="B66" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C66" s="16">
@@ -25882,7 +25882,7 @@
       </c>
       <c r="B67" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C67" s="16">
@@ -25902,7 +25902,7 @@
       </c>
       <c r="B68" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C68" s="16">
@@ -25922,7 +25922,7 @@
       </c>
       <c r="B69" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C69" s="16">
@@ -25942,7 +25942,7 @@
       </c>
       <c r="B70" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C70" s="16">
@@ -26962,7 +26962,7 @@
       </c>
       <c r="B121" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Pipeline Management</t>
         </is>
       </c>
       <c r="C121" s="16">
@@ -26982,7 +26982,7 @@
       </c>
       <c r="B122" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Pipeline Management</t>
         </is>
       </c>
       <c r="C122" s="16">
@@ -27002,7 +27002,7 @@
       </c>
       <c r="B123" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Pipeline Management</t>
         </is>
       </c>
       <c r="C123" s="16">
@@ -27022,7 +27022,7 @@
       </c>
       <c r="B124" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C124" s="16">
@@ -27042,7 +27042,7 @@
       </c>
       <c r="B125" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C125" s="16">
@@ -27062,7 +27062,7 @@
       </c>
       <c r="B126" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C126" s="16">
@@ -27082,7 +27082,7 @@
       </c>
       <c r="B127" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C127" s="16">
@@ -27102,7 +27102,7 @@
       </c>
       <c r="B128" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Pipeline Management</t>
         </is>
       </c>
       <c r="C128" s="16">
@@ -27122,7 +27122,7 @@
       </c>
       <c r="B129" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Pipeline Management</t>
         </is>
       </c>
       <c r="C129" s="16">
@@ -27142,7 +27142,7 @@
       </c>
       <c r="B130" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C130" s="16">
@@ -27162,7 +27162,7 @@
       </c>
       <c r="B131" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C131" s="16">
@@ -27182,7 +27182,7 @@
       </c>
       <c r="B132" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C132" s="16">
@@ -27202,7 +27202,7 @@
       </c>
       <c r="B133" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Integration Support</t>
         </is>
       </c>
       <c r="C133" s="16">
@@ -32456,7 +32456,7 @@
       </c>
       <c r="B111" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Pipeline Management</t>
         </is>
       </c>
       <c r="C111" s="16">
@@ -32486,7 +32486,7 @@
       </c>
       <c r="B112" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Pipeline Management</t>
         </is>
       </c>
       <c r="C112" s="16">
@@ -32512,7 +32512,7 @@
       </c>
       <c r="B113" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Pipeline Management</t>
         </is>
       </c>
       <c r="C113" s="16">
@@ -32538,7 +32538,7 @@
       </c>
       <c r="B114" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Pipeline Management</t>
         </is>
       </c>
       <c r="C114" s="16">
@@ -32568,7 +32568,7 @@
       </c>
       <c r="B115" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Pipeline Management</t>
         </is>
       </c>
       <c r="C115" s="16">
@@ -32594,7 +32594,7 @@
       </c>
       <c r="B116" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Pipeline Management</t>
         </is>
       </c>
       <c r="C116" s="16">
@@ -32620,7 +32620,7 @@
       </c>
       <c r="B117" s="15" t="inlineStr">
         <is>
-          <t>Management</t>
+          <t>Pipeline Management</t>
         </is>
       </c>
       <c r="C117" s="16">

</xml_diff>